<commit_message>
update script and regenerate csvs
script now compiles underlying data and calculates annual effective rate; updated with Dec 2025 trade data
</commit_message>
<xml_diff>
--- a/exh12.xlsx
+++ b/exh12.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\econ019fs\ftd53\TDSB2\Internet\Current\Press-Release\current_press_release\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{71260AD0-2AA1-4C1F-B1DC-59694472284D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2CF0DD33-64CA-48D7-B343-0DBF3F61B52E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8510" yWindow="-10910" windowWidth="19420" windowHeight="10300" xr2:uid="{C18D327F-584E-4CC1-B422-32E4445C5EE3}"/>
+    <workbookView xWindow="8510" yWindow="-10910" windowWidth="19420" windowHeight="10300" xr2:uid="{4216718F-B2CB-490F-B8C0-F1EFDA7AD6A4}"/>
   </bookViews>
   <sheets>
     <sheet name="12" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
     <definedName name="gsfimpcountries">'[2]SF Goods Imports'!$A$4:$S$4</definedName>
     <definedName name="gsfimpquarters">'[2]SF Goods Imports'!$A$4:$A$500</definedName>
     <definedName name="PRINT">#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'12'!$A$1:$I$54</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'12'!$A$1:$I$52</definedName>
     <definedName name="qlookup">[2]Codes!$A$22:$B$25</definedName>
     <definedName name="snsaexp">'[2]NSA Services Exports'!$A$4:$S$500</definedName>
     <definedName name="snsaexpcountries">'[2]NSA Services Exports'!$A$4:$S$4</definedName>
@@ -94,7 +94,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="30">
   <si>
     <t>Part B: NOT Seasonally Adjusted</t>
   </si>
@@ -129,10 +129,7 @@
     <t>2023</t>
   </si>
   <si>
-    <t>Jan. - Dec.</t>
-  </si>
-  <si>
-    <t>Jan. - Nov.</t>
+    <t>Jan.- Dec.</t>
   </si>
   <si>
     <t>January</t>
@@ -177,16 +174,13 @@
     <t>2025</t>
   </si>
   <si>
-    <t>October (R)</t>
+    <t>November (R)</t>
   </si>
   <si>
-    <t/>
+    <t>November data as published last month:</t>
   </si>
   <si>
-    <t>October data as published last month:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOTE: For information on data sources, nonsampling errors, definitions, and details concerning what is included in Net Adjustments, see the explanatory notes in </t>
+    <t>NOTE: For information on data sources, nonsampling errors, definitions, and details concerning what is included in Net Adjustments, see the explanatory notes in</t>
   </si>
   <si>
     <t>this release or at www.census.gov/ft900 or www.bea.gov/data/intl-trade-investment/international-trade-goods-and-services.</t>
@@ -263,7 +257,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="28">
+  <borders count="36">
     <border>
       <left/>
       <right/>
@@ -456,18 +450,11 @@
         <color indexed="8"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color indexed="8"/>
       </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
+      <top style="double">
+        <color indexed="8"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -476,40 +463,35 @@
         <color indexed="8"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color indexed="8"/>
       </right>
-      <top/>
+      <top style="double">
+        <color indexed="8"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
+        <color indexed="8"/>
       </left>
       <right style="double">
         <color indexed="8"/>
       </right>
-      <top/>
+      <top style="double">
+        <color indexed="8"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right style="thin">
-        <color indexed="64"/>
+        <color indexed="8"/>
       </right>
-      <top/>
+      <top style="double">
+        <color indexed="8"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -527,7 +509,7 @@
         <color indexed="8"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color indexed="8"/>
       </right>
       <top/>
       <bottom style="thin">
@@ -537,7 +519,7 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color indexed="8"/>
       </left>
       <right/>
       <top/>
@@ -551,7 +533,7 @@
         <color indexed="8"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color indexed="8"/>
       </right>
       <top/>
       <bottom style="thin">
@@ -561,20 +543,7 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
+        <color indexed="8"/>
       </left>
       <right style="double">
         <color indexed="8"/>
@@ -588,7 +557,7 @@
     <border>
       <left/>
       <right style="thin">
-        <color indexed="64"/>
+        <color indexed="8"/>
       </right>
       <top/>
       <bottom style="thin">
@@ -596,11 +565,132 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color indexed="8"/>
+      </left>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right style="double">
+        <color indexed="8"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color indexed="8"/>
+      </left>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right style="double">
+        <color indexed="8"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -681,37 +771,37 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -56859,203 +56949,200 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{789E9BA0-446B-47D0-8168-9D6BC6CDA87D}">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:HT54"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F58F6FAF-9945-473D-9242-6C3338C549E7}">
+  <dimension ref="A1:HT53"/>
   <sheetFormatPr defaultColWidth="9.69140625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13" style="2" customWidth="1"/>
+    <col min="1" max="1" width="12.69140625" style="2" customWidth="1"/>
     <col min="2" max="9" width="14.69140625" style="2" customWidth="1"/>
     <col min="10" max="256" width="9.69140625" style="4"/>
-    <col min="257" max="257" width="13" style="4" customWidth="1"/>
+    <col min="257" max="257" width="12.69140625" style="4" customWidth="1"/>
     <col min="258" max="265" width="14.69140625" style="4" customWidth="1"/>
     <col min="266" max="512" width="9.69140625" style="4"/>
-    <col min="513" max="513" width="13" style="4" customWidth="1"/>
+    <col min="513" max="513" width="12.69140625" style="4" customWidth="1"/>
     <col min="514" max="521" width="14.69140625" style="4" customWidth="1"/>
     <col min="522" max="768" width="9.69140625" style="4"/>
-    <col min="769" max="769" width="13" style="4" customWidth="1"/>
+    <col min="769" max="769" width="12.69140625" style="4" customWidth="1"/>
     <col min="770" max="777" width="14.69140625" style="4" customWidth="1"/>
     <col min="778" max="1024" width="9.69140625" style="4"/>
-    <col min="1025" max="1025" width="13" style="4" customWidth="1"/>
+    <col min="1025" max="1025" width="12.69140625" style="4" customWidth="1"/>
     <col min="1026" max="1033" width="14.69140625" style="4" customWidth="1"/>
     <col min="1034" max="1280" width="9.69140625" style="4"/>
-    <col min="1281" max="1281" width="13" style="4" customWidth="1"/>
+    <col min="1281" max="1281" width="12.69140625" style="4" customWidth="1"/>
     <col min="1282" max="1289" width="14.69140625" style="4" customWidth="1"/>
     <col min="1290" max="1536" width="9.69140625" style="4"/>
-    <col min="1537" max="1537" width="13" style="4" customWidth="1"/>
+    <col min="1537" max="1537" width="12.69140625" style="4" customWidth="1"/>
     <col min="1538" max="1545" width="14.69140625" style="4" customWidth="1"/>
     <col min="1546" max="1792" width="9.69140625" style="4"/>
-    <col min="1793" max="1793" width="13" style="4" customWidth="1"/>
+    <col min="1793" max="1793" width="12.69140625" style="4" customWidth="1"/>
     <col min="1794" max="1801" width="14.69140625" style="4" customWidth="1"/>
     <col min="1802" max="2048" width="9.69140625" style="4"/>
-    <col min="2049" max="2049" width="13" style="4" customWidth="1"/>
+    <col min="2049" max="2049" width="12.69140625" style="4" customWidth="1"/>
     <col min="2050" max="2057" width="14.69140625" style="4" customWidth="1"/>
     <col min="2058" max="2304" width="9.69140625" style="4"/>
-    <col min="2305" max="2305" width="13" style="4" customWidth="1"/>
+    <col min="2305" max="2305" width="12.69140625" style="4" customWidth="1"/>
     <col min="2306" max="2313" width="14.69140625" style="4" customWidth="1"/>
     <col min="2314" max="2560" width="9.69140625" style="4"/>
-    <col min="2561" max="2561" width="13" style="4" customWidth="1"/>
+    <col min="2561" max="2561" width="12.69140625" style="4" customWidth="1"/>
     <col min="2562" max="2569" width="14.69140625" style="4" customWidth="1"/>
     <col min="2570" max="2816" width="9.69140625" style="4"/>
-    <col min="2817" max="2817" width="13" style="4" customWidth="1"/>
+    <col min="2817" max="2817" width="12.69140625" style="4" customWidth="1"/>
     <col min="2818" max="2825" width="14.69140625" style="4" customWidth="1"/>
     <col min="2826" max="3072" width="9.69140625" style="4"/>
-    <col min="3073" max="3073" width="13" style="4" customWidth="1"/>
+    <col min="3073" max="3073" width="12.69140625" style="4" customWidth="1"/>
     <col min="3074" max="3081" width="14.69140625" style="4" customWidth="1"/>
     <col min="3082" max="3328" width="9.69140625" style="4"/>
-    <col min="3329" max="3329" width="13" style="4" customWidth="1"/>
+    <col min="3329" max="3329" width="12.69140625" style="4" customWidth="1"/>
     <col min="3330" max="3337" width="14.69140625" style="4" customWidth="1"/>
     <col min="3338" max="3584" width="9.69140625" style="4"/>
-    <col min="3585" max="3585" width="13" style="4" customWidth="1"/>
+    <col min="3585" max="3585" width="12.69140625" style="4" customWidth="1"/>
     <col min="3586" max="3593" width="14.69140625" style="4" customWidth="1"/>
     <col min="3594" max="3840" width="9.69140625" style="4"/>
-    <col min="3841" max="3841" width="13" style="4" customWidth="1"/>
+    <col min="3841" max="3841" width="12.69140625" style="4" customWidth="1"/>
     <col min="3842" max="3849" width="14.69140625" style="4" customWidth="1"/>
     <col min="3850" max="4096" width="9.69140625" style="4"/>
-    <col min="4097" max="4097" width="13" style="4" customWidth="1"/>
+    <col min="4097" max="4097" width="12.69140625" style="4" customWidth="1"/>
     <col min="4098" max="4105" width="14.69140625" style="4" customWidth="1"/>
     <col min="4106" max="4352" width="9.69140625" style="4"/>
-    <col min="4353" max="4353" width="13" style="4" customWidth="1"/>
+    <col min="4353" max="4353" width="12.69140625" style="4" customWidth="1"/>
     <col min="4354" max="4361" width="14.69140625" style="4" customWidth="1"/>
     <col min="4362" max="4608" width="9.69140625" style="4"/>
-    <col min="4609" max="4609" width="13" style="4" customWidth="1"/>
+    <col min="4609" max="4609" width="12.69140625" style="4" customWidth="1"/>
     <col min="4610" max="4617" width="14.69140625" style="4" customWidth="1"/>
     <col min="4618" max="4864" width="9.69140625" style="4"/>
-    <col min="4865" max="4865" width="13" style="4" customWidth="1"/>
+    <col min="4865" max="4865" width="12.69140625" style="4" customWidth="1"/>
     <col min="4866" max="4873" width="14.69140625" style="4" customWidth="1"/>
     <col min="4874" max="5120" width="9.69140625" style="4"/>
-    <col min="5121" max="5121" width="13" style="4" customWidth="1"/>
+    <col min="5121" max="5121" width="12.69140625" style="4" customWidth="1"/>
     <col min="5122" max="5129" width="14.69140625" style="4" customWidth="1"/>
     <col min="5130" max="5376" width="9.69140625" style="4"/>
-    <col min="5377" max="5377" width="13" style="4" customWidth="1"/>
+    <col min="5377" max="5377" width="12.69140625" style="4" customWidth="1"/>
     <col min="5378" max="5385" width="14.69140625" style="4" customWidth="1"/>
     <col min="5386" max="5632" width="9.69140625" style="4"/>
-    <col min="5633" max="5633" width="13" style="4" customWidth="1"/>
+    <col min="5633" max="5633" width="12.69140625" style="4" customWidth="1"/>
     <col min="5634" max="5641" width="14.69140625" style="4" customWidth="1"/>
     <col min="5642" max="5888" width="9.69140625" style="4"/>
-    <col min="5889" max="5889" width="13" style="4" customWidth="1"/>
+    <col min="5889" max="5889" width="12.69140625" style="4" customWidth="1"/>
     <col min="5890" max="5897" width="14.69140625" style="4" customWidth="1"/>
     <col min="5898" max="6144" width="9.69140625" style="4"/>
-    <col min="6145" max="6145" width="13" style="4" customWidth="1"/>
+    <col min="6145" max="6145" width="12.69140625" style="4" customWidth="1"/>
     <col min="6146" max="6153" width="14.69140625" style="4" customWidth="1"/>
     <col min="6154" max="6400" width="9.69140625" style="4"/>
-    <col min="6401" max="6401" width="13" style="4" customWidth="1"/>
+    <col min="6401" max="6401" width="12.69140625" style="4" customWidth="1"/>
     <col min="6402" max="6409" width="14.69140625" style="4" customWidth="1"/>
     <col min="6410" max="6656" width="9.69140625" style="4"/>
-    <col min="6657" max="6657" width="13" style="4" customWidth="1"/>
+    <col min="6657" max="6657" width="12.69140625" style="4" customWidth="1"/>
     <col min="6658" max="6665" width="14.69140625" style="4" customWidth="1"/>
     <col min="6666" max="6912" width="9.69140625" style="4"/>
-    <col min="6913" max="6913" width="13" style="4" customWidth="1"/>
+    <col min="6913" max="6913" width="12.69140625" style="4" customWidth="1"/>
     <col min="6914" max="6921" width="14.69140625" style="4" customWidth="1"/>
     <col min="6922" max="7168" width="9.69140625" style="4"/>
-    <col min="7169" max="7169" width="13" style="4" customWidth="1"/>
+    <col min="7169" max="7169" width="12.69140625" style="4" customWidth="1"/>
     <col min="7170" max="7177" width="14.69140625" style="4" customWidth="1"/>
     <col min="7178" max="7424" width="9.69140625" style="4"/>
-    <col min="7425" max="7425" width="13" style="4" customWidth="1"/>
+    <col min="7425" max="7425" width="12.69140625" style="4" customWidth="1"/>
     <col min="7426" max="7433" width="14.69140625" style="4" customWidth="1"/>
     <col min="7434" max="7680" width="9.69140625" style="4"/>
-    <col min="7681" max="7681" width="13" style="4" customWidth="1"/>
+    <col min="7681" max="7681" width="12.69140625" style="4" customWidth="1"/>
     <col min="7682" max="7689" width="14.69140625" style="4" customWidth="1"/>
     <col min="7690" max="7936" width="9.69140625" style="4"/>
-    <col min="7937" max="7937" width="13" style="4" customWidth="1"/>
+    <col min="7937" max="7937" width="12.69140625" style="4" customWidth="1"/>
     <col min="7938" max="7945" width="14.69140625" style="4" customWidth="1"/>
     <col min="7946" max="8192" width="9.69140625" style="4"/>
-    <col min="8193" max="8193" width="13" style="4" customWidth="1"/>
+    <col min="8193" max="8193" width="12.69140625" style="4" customWidth="1"/>
     <col min="8194" max="8201" width="14.69140625" style="4" customWidth="1"/>
     <col min="8202" max="8448" width="9.69140625" style="4"/>
-    <col min="8449" max="8449" width="13" style="4" customWidth="1"/>
+    <col min="8449" max="8449" width="12.69140625" style="4" customWidth="1"/>
     <col min="8450" max="8457" width="14.69140625" style="4" customWidth="1"/>
     <col min="8458" max="8704" width="9.69140625" style="4"/>
-    <col min="8705" max="8705" width="13" style="4" customWidth="1"/>
+    <col min="8705" max="8705" width="12.69140625" style="4" customWidth="1"/>
     <col min="8706" max="8713" width="14.69140625" style="4" customWidth="1"/>
     <col min="8714" max="8960" width="9.69140625" style="4"/>
-    <col min="8961" max="8961" width="13" style="4" customWidth="1"/>
+    <col min="8961" max="8961" width="12.69140625" style="4" customWidth="1"/>
     <col min="8962" max="8969" width="14.69140625" style="4" customWidth="1"/>
     <col min="8970" max="9216" width="9.69140625" style="4"/>
-    <col min="9217" max="9217" width="13" style="4" customWidth="1"/>
+    <col min="9217" max="9217" width="12.69140625" style="4" customWidth="1"/>
     <col min="9218" max="9225" width="14.69140625" style="4" customWidth="1"/>
     <col min="9226" max="9472" width="9.69140625" style="4"/>
-    <col min="9473" max="9473" width="13" style="4" customWidth="1"/>
+    <col min="9473" max="9473" width="12.69140625" style="4" customWidth="1"/>
     <col min="9474" max="9481" width="14.69140625" style="4" customWidth="1"/>
     <col min="9482" max="9728" width="9.69140625" style="4"/>
-    <col min="9729" max="9729" width="13" style="4" customWidth="1"/>
+    <col min="9729" max="9729" width="12.69140625" style="4" customWidth="1"/>
     <col min="9730" max="9737" width="14.69140625" style="4" customWidth="1"/>
     <col min="9738" max="9984" width="9.69140625" style="4"/>
-    <col min="9985" max="9985" width="13" style="4" customWidth="1"/>
+    <col min="9985" max="9985" width="12.69140625" style="4" customWidth="1"/>
     <col min="9986" max="9993" width="14.69140625" style="4" customWidth="1"/>
     <col min="9994" max="10240" width="9.69140625" style="4"/>
-    <col min="10241" max="10241" width="13" style="4" customWidth="1"/>
+    <col min="10241" max="10241" width="12.69140625" style="4" customWidth="1"/>
     <col min="10242" max="10249" width="14.69140625" style="4" customWidth="1"/>
     <col min="10250" max="10496" width="9.69140625" style="4"/>
-    <col min="10497" max="10497" width="13" style="4" customWidth="1"/>
+    <col min="10497" max="10497" width="12.69140625" style="4" customWidth="1"/>
     <col min="10498" max="10505" width="14.69140625" style="4" customWidth="1"/>
     <col min="10506" max="10752" width="9.69140625" style="4"/>
-    <col min="10753" max="10753" width="13" style="4" customWidth="1"/>
+    <col min="10753" max="10753" width="12.69140625" style="4" customWidth="1"/>
     <col min="10754" max="10761" width="14.69140625" style="4" customWidth="1"/>
     <col min="10762" max="11008" width="9.69140625" style="4"/>
-    <col min="11009" max="11009" width="13" style="4" customWidth="1"/>
+    <col min="11009" max="11009" width="12.69140625" style="4" customWidth="1"/>
     <col min="11010" max="11017" width="14.69140625" style="4" customWidth="1"/>
     <col min="11018" max="11264" width="9.69140625" style="4"/>
-    <col min="11265" max="11265" width="13" style="4" customWidth="1"/>
+    <col min="11265" max="11265" width="12.69140625" style="4" customWidth="1"/>
     <col min="11266" max="11273" width="14.69140625" style="4" customWidth="1"/>
     <col min="11274" max="11520" width="9.69140625" style="4"/>
-    <col min="11521" max="11521" width="13" style="4" customWidth="1"/>
+    <col min="11521" max="11521" width="12.69140625" style="4" customWidth="1"/>
     <col min="11522" max="11529" width="14.69140625" style="4" customWidth="1"/>
     <col min="11530" max="11776" width="9.69140625" style="4"/>
-    <col min="11777" max="11777" width="13" style="4" customWidth="1"/>
+    <col min="11777" max="11777" width="12.69140625" style="4" customWidth="1"/>
     <col min="11778" max="11785" width="14.69140625" style="4" customWidth="1"/>
     <col min="11786" max="12032" width="9.69140625" style="4"/>
-    <col min="12033" max="12033" width="13" style="4" customWidth="1"/>
+    <col min="12033" max="12033" width="12.69140625" style="4" customWidth="1"/>
     <col min="12034" max="12041" width="14.69140625" style="4" customWidth="1"/>
     <col min="12042" max="12288" width="9.69140625" style="4"/>
-    <col min="12289" max="12289" width="13" style="4" customWidth="1"/>
+    <col min="12289" max="12289" width="12.69140625" style="4" customWidth="1"/>
     <col min="12290" max="12297" width="14.69140625" style="4" customWidth="1"/>
     <col min="12298" max="12544" width="9.69140625" style="4"/>
-    <col min="12545" max="12545" width="13" style="4" customWidth="1"/>
+    <col min="12545" max="12545" width="12.69140625" style="4" customWidth="1"/>
     <col min="12546" max="12553" width="14.69140625" style="4" customWidth="1"/>
     <col min="12554" max="12800" width="9.69140625" style="4"/>
-    <col min="12801" max="12801" width="13" style="4" customWidth="1"/>
+    <col min="12801" max="12801" width="12.69140625" style="4" customWidth="1"/>
     <col min="12802" max="12809" width="14.69140625" style="4" customWidth="1"/>
     <col min="12810" max="13056" width="9.69140625" style="4"/>
-    <col min="13057" max="13057" width="13" style="4" customWidth="1"/>
+    <col min="13057" max="13057" width="12.69140625" style="4" customWidth="1"/>
     <col min="13058" max="13065" width="14.69140625" style="4" customWidth="1"/>
     <col min="13066" max="13312" width="9.69140625" style="4"/>
-    <col min="13313" max="13313" width="13" style="4" customWidth="1"/>
+    <col min="13313" max="13313" width="12.69140625" style="4" customWidth="1"/>
     <col min="13314" max="13321" width="14.69140625" style="4" customWidth="1"/>
     <col min="13322" max="13568" width="9.69140625" style="4"/>
-    <col min="13569" max="13569" width="13" style="4" customWidth="1"/>
+    <col min="13569" max="13569" width="12.69140625" style="4" customWidth="1"/>
     <col min="13570" max="13577" width="14.69140625" style="4" customWidth="1"/>
     <col min="13578" max="13824" width="9.69140625" style="4"/>
-    <col min="13825" max="13825" width="13" style="4" customWidth="1"/>
+    <col min="13825" max="13825" width="12.69140625" style="4" customWidth="1"/>
     <col min="13826" max="13833" width="14.69140625" style="4" customWidth="1"/>
     <col min="13834" max="14080" width="9.69140625" style="4"/>
-    <col min="14081" max="14081" width="13" style="4" customWidth="1"/>
+    <col min="14081" max="14081" width="12.69140625" style="4" customWidth="1"/>
     <col min="14082" max="14089" width="14.69140625" style="4" customWidth="1"/>
     <col min="14090" max="14336" width="9.69140625" style="4"/>
-    <col min="14337" max="14337" width="13" style="4" customWidth="1"/>
+    <col min="14337" max="14337" width="12.69140625" style="4" customWidth="1"/>
     <col min="14338" max="14345" width="14.69140625" style="4" customWidth="1"/>
     <col min="14346" max="14592" width="9.69140625" style="4"/>
-    <col min="14593" max="14593" width="13" style="4" customWidth="1"/>
+    <col min="14593" max="14593" width="12.69140625" style="4" customWidth="1"/>
     <col min="14594" max="14601" width="14.69140625" style="4" customWidth="1"/>
     <col min="14602" max="14848" width="9.69140625" style="4"/>
-    <col min="14849" max="14849" width="13" style="4" customWidth="1"/>
+    <col min="14849" max="14849" width="12.69140625" style="4" customWidth="1"/>
     <col min="14850" max="14857" width="14.69140625" style="4" customWidth="1"/>
     <col min="14858" max="15104" width="9.69140625" style="4"/>
-    <col min="15105" max="15105" width="13" style="4" customWidth="1"/>
+    <col min="15105" max="15105" width="12.69140625" style="4" customWidth="1"/>
     <col min="15106" max="15113" width="14.69140625" style="4" customWidth="1"/>
     <col min="15114" max="15360" width="9.69140625" style="4"/>
-    <col min="15361" max="15361" width="13" style="4" customWidth="1"/>
+    <col min="15361" max="15361" width="12.69140625" style="4" customWidth="1"/>
     <col min="15362" max="15369" width="14.69140625" style="4" customWidth="1"/>
     <col min="15370" max="15616" width="9.69140625" style="4"/>
-    <col min="15617" max="15617" width="13" style="4" customWidth="1"/>
+    <col min="15617" max="15617" width="12.69140625" style="4" customWidth="1"/>
     <col min="15618" max="15625" width="14.69140625" style="4" customWidth="1"/>
     <col min="15626" max="15872" width="9.69140625" style="4"/>
-    <col min="15873" max="15873" width="13" style="4" customWidth="1"/>
+    <col min="15873" max="15873" width="12.69140625" style="4" customWidth="1"/>
     <col min="15874" max="15881" width="14.69140625" style="4" customWidth="1"/>
     <col min="15882" max="16128" width="9.69140625" style="4"/>
-    <col min="16129" max="16129" width="13" style="4" customWidth="1"/>
+    <col min="16129" max="16129" width="12.69140625" style="4" customWidth="1"/>
     <col min="16130" max="16137" width="14.69140625" style="4" customWidth="1"/>
     <col min="16138" max="16384" width="9.69140625" style="4"/>
   </cols>
@@ -57594,14 +57681,14 @@
       <c r="B7" s="29"/>
       <c r="C7" s="30"/>
       <c r="D7" s="31"/>
-      <c r="E7" s="32"/>
-      <c r="F7" s="33"/>
-      <c r="G7" s="34"/>
-      <c r="H7" s="32"/>
+      <c r="E7" s="29"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="33"/>
+      <c r="H7" s="29"/>
       <c r="I7" s="30"/>
     </row>
     <row r="8" spans="1:228" ht="25.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="34" t="s">
         <v>11</v>
       </c>
       <c r="B8" s="35">
@@ -57613,1256 +57700,1199 @@
       <c r="D8" s="37">
         <v>2047457</v>
       </c>
-      <c r="E8" s="38">
+      <c r="E8" s="35">
         <v>26978</v>
       </c>
-      <c r="F8" s="39">
+      <c r="F8" s="38">
         <v>2020479</v>
       </c>
-      <c r="G8" s="40">
+      <c r="G8" s="39">
         <v>3104952</v>
       </c>
-      <c r="H8" s="38">
+      <c r="H8" s="35">
         <v>28155</v>
       </c>
       <c r="I8" s="36">
         <v>3076796</v>
       </c>
     </row>
-    <row r="9" spans="1:228" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="41" t="s">
+    <row r="9" spans="1:228" ht="22.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="42">
-        <v>-977234</v>
+      <c r="B9" s="40">
+        <v>-90826</v>
       </c>
-      <c r="C9" s="43">
-        <v>-976968</v>
+      <c r="C9" s="41">
+        <v>-89854</v>
       </c>
-      <c r="D9" s="44">
-        <v>1878348</v>
+      <c r="D9" s="42">
+        <v>166188</v>
       </c>
-      <c r="E9" s="45">
-        <v>25560</v>
+      <c r="E9" s="40">
+        <v>1416</v>
       </c>
-      <c r="F9" s="46">
-        <v>1852788</v>
+      <c r="F9" s="43">
+        <v>164772</v>
       </c>
-      <c r="G9" s="47">
-        <v>2855582</v>
+      <c r="G9" s="44">
+        <v>257014</v>
       </c>
-      <c r="H9" s="45">
-        <v>25827</v>
+      <c r="H9" s="40">
+        <v>2388</v>
       </c>
-      <c r="I9" s="43">
-        <v>2829755</v>
+      <c r="I9" s="41">
+        <v>254626</v>
       </c>
     </row>
-    <row r="10" spans="1:228" ht="22.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:228" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="35">
-        <v>-90826</v>
+      <c r="B10" s="40">
+        <v>-72282</v>
       </c>
-      <c r="C10" s="36">
-        <v>-89854</v>
+      <c r="C10" s="41">
+        <v>-71449</v>
       </c>
-      <c r="D10" s="37">
-        <v>166188</v>
+      <c r="D10" s="42">
+        <v>160255</v>
       </c>
-      <c r="E10" s="38">
-        <v>1416</v>
+      <c r="E10" s="40">
+        <v>1533</v>
       </c>
-      <c r="F10" s="39">
-        <v>164772</v>
+      <c r="F10" s="43">
+        <v>158721</v>
       </c>
-      <c r="G10" s="40">
-        <v>257014</v>
+      <c r="G10" s="44">
+        <v>232536</v>
       </c>
-      <c r="H10" s="38">
-        <v>2388</v>
+      <c r="H10" s="40">
+        <v>2367</v>
       </c>
-      <c r="I10" s="36">
-        <v>254626</v>
+      <c r="I10" s="41">
+        <v>230170</v>
       </c>
     </row>
     <row r="11" spans="1:228" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="35">
-        <v>-72282</v>
+      <c r="B11" s="40">
+        <v>-78355</v>
       </c>
-      <c r="C11" s="36">
-        <v>-71449</v>
+      <c r="C11" s="41">
+        <v>-77673</v>
       </c>
-      <c r="D11" s="37">
-        <v>160255</v>
+      <c r="D11" s="42">
+        <v>185455</v>
       </c>
-      <c r="E11" s="38">
-        <v>1533</v>
+      <c r="E11" s="40">
+        <v>1884</v>
       </c>
-      <c r="F11" s="39">
-        <v>158721</v>
+      <c r="F11" s="43">
+        <v>183571</v>
       </c>
-      <c r="G11" s="40">
-        <v>232536</v>
+      <c r="G11" s="44">
+        <v>263809</v>
       </c>
-      <c r="H11" s="38">
-        <v>2367</v>
+      <c r="H11" s="40">
+        <v>2566</v>
       </c>
-      <c r="I11" s="36">
-        <v>230170</v>
+      <c r="I11" s="41">
+        <v>261244</v>
       </c>
     </row>
     <row r="12" spans="1:228" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="35">
-        <v>-78355</v>
+      <c r="B12" s="40">
+        <v>-86853</v>
       </c>
-      <c r="C12" s="36">
-        <v>-77673</v>
+      <c r="C12" s="41">
+        <v>-87204</v>
       </c>
-      <c r="D12" s="37">
-        <v>185455</v>
+      <c r="D12" s="42">
+        <v>165282</v>
       </c>
-      <c r="E12" s="38">
-        <v>1884</v>
+      <c r="E12" s="40">
+        <v>2617</v>
       </c>
-      <c r="F12" s="39">
-        <v>183571</v>
+      <c r="F12" s="43">
+        <v>162666</v>
       </c>
-      <c r="G12" s="40">
-        <v>263809</v>
+      <c r="G12" s="44">
+        <v>252135</v>
       </c>
-      <c r="H12" s="38">
-        <v>2566</v>
+      <c r="H12" s="40">
+        <v>2266</v>
       </c>
-      <c r="I12" s="36">
-        <v>261244</v>
+      <c r="I12" s="41">
+        <v>249869</v>
       </c>
     </row>
     <row r="13" spans="1:228" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="35">
-        <v>-86853</v>
+      <c r="B13" s="40">
+        <v>-95667</v>
       </c>
-      <c r="C13" s="36">
-        <v>-87204</v>
+      <c r="C13" s="41">
+        <v>-96101</v>
       </c>
-      <c r="D13" s="37">
-        <v>165282</v>
+      <c r="D13" s="42">
+        <v>169763</v>
       </c>
-      <c r="E13" s="38">
-        <v>2617</v>
+      <c r="E13" s="40">
+        <v>2619</v>
       </c>
-      <c r="F13" s="39">
-        <v>162666</v>
+      <c r="F13" s="43">
+        <v>167144</v>
       </c>
-      <c r="G13" s="40">
-        <v>252135</v>
+      <c r="G13" s="44">
+        <v>265430</v>
       </c>
-      <c r="H13" s="38">
-        <v>2266</v>
+      <c r="H13" s="40">
+        <v>2185</v>
       </c>
-      <c r="I13" s="36">
-        <v>249869</v>
+      <c r="I13" s="41">
+        <v>263245</v>
       </c>
     </row>
     <row r="14" spans="1:228" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="35">
-        <v>-95667</v>
+      <c r="B14" s="40">
+        <v>-89752</v>
       </c>
-      <c r="C14" s="36">
-        <v>-96101</v>
+      <c r="C14" s="41">
+        <v>-90057</v>
       </c>
-      <c r="D14" s="37">
-        <v>169763</v>
+      <c r="D14" s="42">
+        <v>169483</v>
       </c>
-      <c r="E14" s="38">
-        <v>2619</v>
+      <c r="E14" s="40">
+        <v>2329</v>
       </c>
-      <c r="F14" s="39">
-        <v>167144</v>
+      <c r="F14" s="43">
+        <v>167154</v>
       </c>
-      <c r="G14" s="40">
-        <v>265430</v>
+      <c r="G14" s="44">
+        <v>259235</v>
       </c>
-      <c r="H14" s="38">
-        <v>2185</v>
+      <c r="H14" s="40">
+        <v>2024</v>
       </c>
-      <c r="I14" s="36">
-        <v>263245</v>
+      <c r="I14" s="41">
+        <v>257211</v>
       </c>
     </row>
-    <row r="15" spans="1:228" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:228" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="35">
-        <v>-89752</v>
+      <c r="B15" s="40">
+        <v>-94321</v>
       </c>
-      <c r="C15" s="36">
-        <v>-90057</v>
+      <c r="C15" s="41">
+        <v>-95135</v>
       </c>
-      <c r="D15" s="37">
-        <v>169483</v>
+      <c r="D15" s="42">
+        <v>163123</v>
       </c>
-      <c r="E15" s="38">
-        <v>2329</v>
+      <c r="E15" s="40">
+        <v>2925</v>
       </c>
-      <c r="F15" s="39">
-        <v>167154</v>
+      <c r="F15" s="43">
+        <v>160198</v>
       </c>
-      <c r="G15" s="40">
-        <v>259235</v>
+      <c r="G15" s="44">
+        <v>257444</v>
       </c>
-      <c r="H15" s="38">
-        <v>2024</v>
+      <c r="H15" s="40">
+        <v>2111</v>
       </c>
-      <c r="I15" s="36">
-        <v>257211</v>
+      <c r="I15" s="41">
+        <v>255333</v>
       </c>
     </row>
-    <row r="16" spans="1:228" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:228" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="35">
-        <v>-94321</v>
+      <c r="B16" s="40">
+        <v>-92922</v>
       </c>
-      <c r="C16" s="36">
-        <v>-95135</v>
+      <c r="C16" s="41">
+        <v>-92865</v>
       </c>
-      <c r="D16" s="37">
-        <v>163123</v>
+      <c r="D16" s="42">
+        <v>175172</v>
       </c>
-      <c r="E16" s="38">
-        <v>2925</v>
+      <c r="E16" s="40">
+        <v>2481</v>
       </c>
-      <c r="F16" s="39">
-        <v>160198</v>
+      <c r="F16" s="43">
+        <v>172691</v>
       </c>
-      <c r="G16" s="40">
-        <v>257444</v>
+      <c r="G16" s="44">
+        <v>268094</v>
       </c>
-      <c r="H16" s="38">
-        <v>2111</v>
+      <c r="H16" s="40">
+        <v>2538</v>
       </c>
-      <c r="I16" s="36">
-        <v>255333</v>
+      <c r="I16" s="41">
+        <v>265555</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="35">
-        <v>-92922</v>
+      <c r="B17" s="40">
+        <v>-88664</v>
       </c>
-      <c r="C17" s="36">
-        <v>-92865</v>
+      <c r="C17" s="41">
+        <v>-88973</v>
       </c>
-      <c r="D17" s="37">
-        <v>175172</v>
+      <c r="D17" s="42">
+        <v>174617</v>
       </c>
-      <c r="E17" s="38">
-        <v>2481</v>
+      <c r="E17" s="40">
+        <v>2727</v>
       </c>
-      <c r="F17" s="39">
-        <v>172691</v>
+      <c r="F17" s="43">
+        <v>171890</v>
       </c>
-      <c r="G17" s="40">
-        <v>268094</v>
+      <c r="G17" s="44">
+        <v>263281</v>
       </c>
-      <c r="H17" s="38">
-        <v>2538</v>
+      <c r="H17" s="40">
+        <v>2418</v>
       </c>
-      <c r="I17" s="36">
-        <v>265555</v>
+      <c r="I17" s="41">
+        <v>260863</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="35">
-        <v>-88664</v>
+      <c r="B18" s="40">
+        <v>-98078</v>
       </c>
-      <c r="C18" s="36">
-        <v>-88973</v>
+      <c r="C18" s="41">
+        <v>-97842</v>
       </c>
-      <c r="D18" s="37">
-        <v>174617</v>
+      <c r="D18" s="42">
+        <v>180665</v>
       </c>
-      <c r="E18" s="38">
-        <v>2727</v>
+      <c r="E18" s="40">
+        <v>2329</v>
       </c>
-      <c r="F18" s="39">
-        <v>171890</v>
+      <c r="F18" s="43">
+        <v>178336</v>
       </c>
-      <c r="G18" s="40">
-        <v>263281</v>
+      <c r="G18" s="44">
+        <v>278743</v>
       </c>
-      <c r="H18" s="38">
-        <v>2418</v>
+      <c r="H18" s="40">
+        <v>2565</v>
       </c>
-      <c r="I18" s="36">
-        <v>260863</v>
+      <c r="I18" s="41">
+        <v>276179</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="35">
-        <v>-98078</v>
+      <c r="B19" s="40">
+        <v>-89514</v>
       </c>
-      <c r="C19" s="36">
-        <v>-97842</v>
+      <c r="C19" s="41">
+        <v>-89816</v>
       </c>
-      <c r="D19" s="37">
-        <v>180665</v>
+      <c r="D19" s="42">
+        <v>168346</v>
       </c>
-      <c r="E19" s="38">
-        <v>2329</v>
+      <c r="E19" s="40">
+        <v>2701</v>
       </c>
-      <c r="F19" s="39">
-        <v>178336</v>
+      <c r="F19" s="43">
+        <v>165646</v>
       </c>
-      <c r="G19" s="40">
-        <v>278743</v>
+      <c r="G19" s="44">
+        <v>257861</v>
       </c>
-      <c r="H19" s="38">
-        <v>2565</v>
+      <c r="H19" s="40">
+        <v>2399</v>
       </c>
-      <c r="I19" s="36">
-        <v>276179</v>
+      <c r="I19" s="41">
+        <v>255461</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="35">
-        <v>-89514</v>
-      </c>
-      <c r="C20" s="36">
-        <v>-89816</v>
-      </c>
-      <c r="D20" s="37">
-        <v>168346</v>
-      </c>
-      <c r="E20" s="38">
-        <v>2701</v>
-      </c>
-      <c r="F20" s="39">
-        <v>165646</v>
-      </c>
-      <c r="G20" s="40">
-        <v>257861</v>
-      </c>
-      <c r="H20" s="38">
-        <v>2399</v>
-      </c>
-      <c r="I20" s="36">
-        <v>255461</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B21" s="35">
+      <c r="B20" s="40">
         <v>-80261</v>
       </c>
-      <c r="C21" s="36">
+      <c r="C20" s="41">
         <v>-79350</v>
       </c>
-      <c r="D21" s="37">
+      <c r="D20" s="42">
         <v>169109</v>
       </c>
-      <c r="E21" s="38">
+      <c r="E20" s="40">
         <v>1418</v>
       </c>
-      <c r="F21" s="39">
+      <c r="F20" s="43">
         <v>167692</v>
       </c>
-      <c r="G21" s="40">
+      <c r="G20" s="44">
         <v>249370</v>
       </c>
-      <c r="H21" s="38">
+      <c r="H20" s="40">
         <v>2329</v>
       </c>
-      <c r="I21" s="36">
+      <c r="I20" s="41">
         <v>247041</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="48" t="s">
-        <v>25</v>
+    <row r="21" spans="1:9" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="45" t="s">
+        <v>24</v>
       </c>
-      <c r="B22" s="35"/>
-      <c r="C22" s="36"/>
-      <c r="D22" s="37"/>
-      <c r="E22" s="38"/>
-      <c r="F22" s="39"/>
-      <c r="G22" s="40"/>
-      <c r="H22" s="38"/>
-      <c r="I22" s="36"/>
+      <c r="B21" s="40"/>
+      <c r="C21" s="41"/>
+      <c r="D21" s="42"/>
+      <c r="E21" s="40"/>
+      <c r="F21" s="43"/>
+      <c r="G21" s="44"/>
+      <c r="H21" s="40"/>
+      <c r="I21" s="41"/>
     </row>
-    <row r="23" spans="1:9" ht="25.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="2" t="s">
+    <row r="22" spans="1:9" ht="25.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="B23" s="35">
+      <c r="B22" s="35">
         <v>-1215403</v>
       </c>
-      <c r="C23" s="36">
+      <c r="C22" s="36">
         <v>-1204719</v>
       </c>
-      <c r="D23" s="37">
+      <c r="D22" s="37">
         <v>2079777</v>
       </c>
-      <c r="E23" s="38">
+      <c r="E22" s="35">
         <v>18086</v>
       </c>
-      <c r="F23" s="39">
+      <c r="F22" s="38">
         <v>2061691</v>
       </c>
-      <c r="G23" s="40">
+      <c r="G22" s="39">
         <v>3295180</v>
       </c>
-      <c r="H23" s="38">
+      <c r="H22" s="35">
         <v>28770</v>
       </c>
-      <c r="I23" s="36">
+      <c r="I22" s="36">
         <v>3266410</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="14.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="41" t="s">
+    <row r="23" spans="1:9" ht="22.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B24" s="42">
-        <v>-1095322</v>
+      <c r="B23" s="40">
+        <v>-94963</v>
       </c>
-      <c r="C24" s="43">
-        <v>-1085167</v>
+      <c r="C23" s="41">
+        <v>-93527</v>
       </c>
-      <c r="D24" s="44">
-        <v>1912583</v>
+      <c r="D23" s="42">
+        <v>161408</v>
       </c>
-      <c r="E24" s="45">
-        <v>16251</v>
+      <c r="E23" s="40">
+        <v>1242</v>
       </c>
-      <c r="F24" s="46">
-        <v>1896332</v>
+      <c r="F23" s="43">
+        <v>160165</v>
       </c>
-      <c r="G24" s="47">
-        <v>3007905</v>
+      <c r="G23" s="44">
+        <v>256370</v>
       </c>
-      <c r="H24" s="45">
-        <v>26406</v>
+      <c r="H23" s="40">
+        <v>2678</v>
       </c>
-      <c r="I24" s="43">
-        <v>2981499</v>
+      <c r="I23" s="41">
+        <v>253693</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="22.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="2" t="s">
+    <row r="24" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B25" s="35">
-        <v>-94963</v>
+      <c r="B24" s="40">
+        <v>-76098</v>
       </c>
-      <c r="C25" s="36">
-        <v>-93527</v>
+      <c r="C24" s="41">
+        <v>-74766</v>
       </c>
-      <c r="D25" s="37">
-        <v>161408</v>
+      <c r="D24" s="42">
+        <v>168673</v>
       </c>
-      <c r="E25" s="38">
-        <v>1242</v>
+      <c r="E24" s="40">
+        <v>1209</v>
       </c>
-      <c r="F25" s="39">
-        <v>160165</v>
+      <c r="F24" s="43">
+        <v>167464</v>
       </c>
-      <c r="G25" s="40">
-        <v>256370</v>
+      <c r="G24" s="44">
+        <v>244771</v>
       </c>
-      <c r="H25" s="38">
-        <v>2678</v>
+      <c r="H24" s="40">
+        <v>2541</v>
       </c>
-      <c r="I25" s="36">
-        <v>253693</v>
+      <c r="I24" s="41">
+        <v>242229</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B25" s="40">
+        <v>-80838</v>
+      </c>
+      <c r="C25" s="41">
+        <v>-79717</v>
+      </c>
+      <c r="D25" s="42">
+        <v>180601</v>
+      </c>
+      <c r="E25" s="40">
+        <v>1232</v>
+      </c>
+      <c r="F25" s="43">
+        <v>179370</v>
+      </c>
+      <c r="G25" s="44">
+        <v>261440</v>
+      </c>
+      <c r="H25" s="40">
+        <v>2353</v>
+      </c>
+      <c r="I25" s="41">
+        <v>259087</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
-      <c r="B26" s="35">
-        <v>-76098</v>
+      <c r="B26" s="40">
+        <v>-101443</v>
       </c>
-      <c r="C26" s="36">
-        <v>-74766</v>
+      <c r="C26" s="41">
+        <v>-99824</v>
       </c>
-      <c r="D26" s="37">
-        <v>168673</v>
+      <c r="D26" s="42">
+        <v>172212</v>
       </c>
-      <c r="E26" s="38">
-        <v>1209</v>
+      <c r="E26" s="40">
+        <v>1062</v>
       </c>
-      <c r="F26" s="39">
-        <v>167464</v>
+      <c r="F26" s="43">
+        <v>171150</v>
       </c>
-      <c r="G26" s="40">
-        <v>244771</v>
+      <c r="G26" s="44">
+        <v>273655</v>
       </c>
-      <c r="H26" s="38">
-        <v>2541</v>
+      <c r="H26" s="40">
+        <v>2681</v>
       </c>
-      <c r="I26" s="36">
-        <v>242229</v>
+      <c r="I26" s="41">
+        <v>270974</v>
       </c>
     </row>
     <row r="27" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
-      <c r="B27" s="35">
-        <v>-80838</v>
+      <c r="B27" s="40">
+        <v>-103085</v>
       </c>
-      <c r="C27" s="36">
-        <v>-79717</v>
+      <c r="C27" s="41">
+        <v>-101861</v>
       </c>
-      <c r="D27" s="37">
-        <v>180601</v>
+      <c r="D27" s="42">
+        <v>174523</v>
       </c>
-      <c r="E27" s="38">
-        <v>1232</v>
+      <c r="E27" s="40">
+        <v>1477</v>
       </c>
-      <c r="F27" s="39">
-        <v>179370</v>
+      <c r="F27" s="43">
+        <v>173045</v>
       </c>
-      <c r="G27" s="40">
-        <v>261440</v>
+      <c r="G27" s="44">
+        <v>277608</v>
       </c>
-      <c r="H27" s="38">
-        <v>2353</v>
+      <c r="H27" s="40">
+        <v>2701</v>
       </c>
-      <c r="I27" s="36">
-        <v>259087</v>
+      <c r="I27" s="41">
+        <v>274906</v>
       </c>
     </row>
     <row r="28" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
-      <c r="B28" s="35">
-        <v>-101443</v>
+      <c r="B28" s="40">
+        <v>-92811</v>
       </c>
-      <c r="C28" s="36">
-        <v>-99824</v>
+      <c r="C28" s="41">
+        <v>-92076</v>
       </c>
-      <c r="D28" s="37">
-        <v>172212</v>
+      <c r="D28" s="42">
+        <v>175271</v>
       </c>
-      <c r="E28" s="38">
-        <v>1062</v>
+      <c r="E28" s="40">
+        <v>1290</v>
       </c>
-      <c r="F28" s="39">
-        <v>171150</v>
+      <c r="F28" s="43">
+        <v>173980</v>
       </c>
-      <c r="G28" s="40">
-        <v>273655</v>
+      <c r="G28" s="44">
+        <v>268081</v>
       </c>
-      <c r="H28" s="38">
-        <v>2681</v>
+      <c r="H28" s="40">
+        <v>2025</v>
       </c>
-      <c r="I28" s="36">
-        <v>270974</v>
+      <c r="I28" s="41">
+        <v>266057</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
-      <c r="B29" s="35">
-        <v>-103085</v>
+      <c r="B29" s="40">
+        <v>-119632</v>
       </c>
-      <c r="C29" s="36">
-        <v>-101861</v>
+      <c r="C29" s="41">
+        <v>-119239</v>
       </c>
-      <c r="D29" s="37">
-        <v>174523</v>
+      <c r="D29" s="42">
+        <v>170798</v>
       </c>
-      <c r="E29" s="38">
-        <v>1477</v>
+      <c r="E29" s="40">
+        <v>1910</v>
       </c>
-      <c r="F29" s="39">
-        <v>173045</v>
+      <c r="F29" s="43">
+        <v>168888</v>
       </c>
-      <c r="G29" s="40">
-        <v>277608</v>
+      <c r="G29" s="44">
+        <v>290430</v>
       </c>
-      <c r="H29" s="38">
-        <v>2701</v>
+      <c r="H29" s="40">
+        <v>2303</v>
       </c>
-      <c r="I29" s="36">
-        <v>274906</v>
+      <c r="I29" s="41">
+        <v>288127</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
-      <c r="B30" s="35">
-        <v>-92811</v>
+      <c r="B30" s="40">
+        <v>-98273</v>
       </c>
-      <c r="C30" s="36">
-        <v>-92076</v>
+      <c r="C30" s="41">
+        <v>-97157</v>
       </c>
-      <c r="D30" s="37">
-        <v>175271</v>
+      <c r="D30" s="42">
+        <v>181425</v>
       </c>
-      <c r="E30" s="38">
-        <v>1290</v>
+      <c r="E30" s="40">
+        <v>1275</v>
       </c>
-      <c r="F30" s="39">
-        <v>173980</v>
+      <c r="F30" s="43">
+        <v>180150</v>
       </c>
-      <c r="G30" s="40">
-        <v>268081</v>
+      <c r="G30" s="44">
+        <v>279698</v>
       </c>
-      <c r="H30" s="38">
-        <v>2025</v>
+      <c r="H30" s="40">
+        <v>2392</v>
       </c>
-      <c r="I30" s="36">
-        <v>266057</v>
+      <c r="I30" s="41">
+        <v>277306</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
-      <c r="B31" s="35">
-        <v>-119632</v>
+      <c r="B31" s="40">
+        <v>-115315</v>
       </c>
-      <c r="C31" s="36">
-        <v>-119239</v>
+      <c r="C31" s="41">
+        <v>-114627</v>
       </c>
-      <c r="D31" s="37">
-        <v>170798</v>
+      <c r="D31" s="42">
+        <v>172864</v>
       </c>
-      <c r="E31" s="38">
-        <v>1910</v>
+      <c r="E31" s="40">
+        <v>1527</v>
       </c>
-      <c r="F31" s="39">
-        <v>168888</v>
+      <c r="F31" s="43">
+        <v>171336</v>
       </c>
-      <c r="G31" s="40">
-        <v>290430</v>
+      <c r="G31" s="44">
+        <v>288178</v>
       </c>
-      <c r="H31" s="38">
-        <v>2303</v>
+      <c r="H31" s="40">
+        <v>2215</v>
       </c>
-      <c r="I31" s="36">
-        <v>288127</v>
+      <c r="I31" s="41">
+        <v>285963</v>
       </c>
     </row>
     <row r="32" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
-      <c r="B32" s="35">
-        <v>-98273</v>
+      <c r="B32" s="46">
+        <v>-112795</v>
       </c>
-      <c r="C32" s="36">
-        <v>-97157</v>
+      <c r="C32" s="47">
+        <v>-112099</v>
       </c>
-      <c r="D32" s="37">
-        <v>181425</v>
+      <c r="D32" s="42">
+        <v>178466</v>
       </c>
-      <c r="E32" s="38">
-        <v>1275</v>
+      <c r="E32" s="46">
+        <v>1720</v>
       </c>
-      <c r="F32" s="39">
-        <v>180150</v>
+      <c r="F32" s="48">
+        <v>176745</v>
       </c>
-      <c r="G32" s="40">
-        <v>279698</v>
+      <c r="G32" s="44">
+        <v>291261</v>
       </c>
-      <c r="H32" s="38">
-        <v>2392</v>
+      <c r="H32" s="46">
+        <v>2417</v>
       </c>
-      <c r="I32" s="36">
-        <v>277306</v>
+      <c r="I32" s="47">
+        <v>288844</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
-      <c r="B33" s="35">
-        <v>-115315</v>
+      <c r="B33" s="40">
+        <v>-100069</v>
       </c>
-      <c r="C33" s="36">
-        <v>-114627</v>
+      <c r="C33" s="41">
+        <v>-100274</v>
       </c>
-      <c r="D33" s="37">
-        <v>172864</v>
+      <c r="D33" s="42">
+        <v>176344</v>
       </c>
-      <c r="E33" s="38">
-        <v>1527</v>
+      <c r="E33" s="40">
+        <v>2305</v>
       </c>
-      <c r="F33" s="39">
-        <v>171336</v>
+      <c r="F33" s="43">
+        <v>174038</v>
       </c>
-      <c r="G33" s="40">
-        <v>288178</v>
+      <c r="G33" s="44">
+        <v>276413</v>
       </c>
-      <c r="H33" s="38">
-        <v>2215</v>
+      <c r="H33" s="40">
+        <v>2101</v>
       </c>
-      <c r="I33" s="36">
-        <v>285963</v>
+      <c r="I33" s="41">
+        <v>274312</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B34" s="49">
-        <v>-112795</v>
-      </c>
-      <c r="C34" s="50">
-        <v>-112099</v>
-      </c>
-      <c r="D34" s="37">
-        <v>178466</v>
-      </c>
-      <c r="E34" s="51">
-        <v>1720</v>
-      </c>
-      <c r="F34" s="52">
-        <v>176745</v>
-      </c>
-      <c r="G34" s="40">
-        <v>291261</v>
-      </c>
-      <c r="H34" s="51">
-        <v>2417</v>
-      </c>
-      <c r="I34" s="50">
-        <v>288844</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B35" s="35">
-        <v>-100069</v>
-      </c>
-      <c r="C35" s="36">
-        <v>-100274</v>
-      </c>
-      <c r="D35" s="37">
-        <v>176344</v>
-      </c>
-      <c r="E35" s="38">
-        <v>2305</v>
-      </c>
-      <c r="F35" s="39">
-        <v>174038</v>
-      </c>
-      <c r="G35" s="40">
-        <v>276413</v>
-      </c>
-      <c r="H35" s="38">
-        <v>2101</v>
-      </c>
-      <c r="I35" s="36">
-        <v>274312</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B36" s="35">
+      <c r="B34" s="40">
         <v>-120081</v>
       </c>
-      <c r="C36" s="36">
+      <c r="C34" s="41">
         <v>-119553</v>
       </c>
-      <c r="D36" s="37">
+      <c r="D34" s="42">
         <v>167194</v>
       </c>
-      <c r="E36" s="38">
+      <c r="E34" s="40">
         <v>1836</v>
       </c>
-      <c r="F36" s="39">
+      <c r="F34" s="43">
         <v>165358</v>
       </c>
-      <c r="G36" s="40">
+      <c r="G34" s="44">
         <v>287275</v>
       </c>
-      <c r="H36" s="38">
+      <c r="H34" s="40">
         <v>2363</v>
       </c>
-      <c r="I36" s="36">
+      <c r="I34" s="41">
         <v>284911</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="48" t="s">
-        <v>26</v>
+    <row r="35" spans="1:9" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="45" t="s">
+        <v>25</v>
       </c>
-      <c r="B37" s="35"/>
-      <c r="C37" s="36"/>
-      <c r="D37" s="37"/>
-      <c r="E37" s="38"/>
-      <c r="F37" s="39"/>
-      <c r="G37" s="40"/>
-      <c r="H37" s="38"/>
-      <c r="I37" s="36"/>
+      <c r="B35" s="40"/>
+      <c r="C35" s="41"/>
+      <c r="D35" s="42"/>
+      <c r="E35" s="40"/>
+      <c r="F35" s="43"/>
+      <c r="G35" s="44"/>
+      <c r="H35" s="40"/>
+      <c r="I35" s="41"/>
     </row>
-    <row r="38" spans="1:9" ht="24.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="41" t="s">
+    <row r="36" spans="1:9" ht="25.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="34" t="s">
+        <v>11</v>
+      </c>
+      <c r="B36" s="35">
+        <v>-1240941</v>
+      </c>
+      <c r="C36" s="36">
+        <v>-1230513</v>
+      </c>
+      <c r="D36" s="37">
+        <v>2197486</v>
+      </c>
+      <c r="E36" s="35">
+        <v>12266</v>
+      </c>
+      <c r="F36" s="38">
+        <v>2185220</v>
+      </c>
+      <c r="G36" s="39">
+        <v>3438427</v>
+      </c>
+      <c r="H36" s="35">
+        <v>22695</v>
+      </c>
+      <c r="I36" s="36">
+        <v>3415733</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="22.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B38" s="42">
-        <v>-1139717</v>
+      <c r="B37" s="40">
+        <v>-153278</v>
       </c>
-      <c r="C38" s="43">
-        <v>-1130047</v>
+      <c r="C37" s="41">
+        <v>-152364</v>
       </c>
-      <c r="D38" s="44">
-        <v>2016684</v>
+      <c r="D37" s="42">
+        <v>165893</v>
       </c>
-      <c r="E38" s="45">
-        <v>11489</v>
+      <c r="E37" s="40">
+        <v>1031</v>
       </c>
-      <c r="F38" s="46">
-        <v>2005196</v>
+      <c r="F37" s="43">
+        <v>164862</v>
       </c>
-      <c r="G38" s="47">
-        <v>3156401</v>
+      <c r="G37" s="44">
+        <v>319171</v>
       </c>
-      <c r="H38" s="45">
-        <v>21159</v>
+      <c r="H37" s="40">
+        <v>1944</v>
       </c>
-      <c r="I38" s="43">
-        <v>3135242</v>
+      <c r="I37" s="41">
+        <v>317227</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="22.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="2" t="s">
+    <row r="38" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B39" s="35">
-        <v>-153278</v>
+      <c r="B38" s="40">
+        <v>-119801</v>
       </c>
-      <c r="C39" s="36">
-        <v>-152364</v>
+      <c r="C38" s="41">
+        <v>-120619</v>
       </c>
-      <c r="D39" s="37">
-        <v>165893</v>
+      <c r="D38" s="42">
+        <v>170423</v>
       </c>
-      <c r="E39" s="38">
-        <v>1031</v>
+      <c r="E38" s="40">
+        <v>2848</v>
       </c>
-      <c r="F39" s="39">
-        <v>164862</v>
+      <c r="F38" s="43">
+        <v>167575</v>
       </c>
-      <c r="G39" s="40">
-        <v>319171</v>
+      <c r="G38" s="44">
+        <v>290224</v>
       </c>
-      <c r="H39" s="38">
-        <v>1944</v>
+      <c r="H38" s="40">
+        <v>2030</v>
       </c>
-      <c r="I39" s="36">
-        <v>317227</v>
+      <c r="I38" s="41">
+        <v>288194</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B39" s="40">
+        <v>-151950</v>
+      </c>
+      <c r="C39" s="41">
+        <v>-151316</v>
+      </c>
+      <c r="D39" s="42">
+        <v>192967</v>
+      </c>
+      <c r="E39" s="40">
+        <v>1556</v>
+      </c>
+      <c r="F39" s="43">
+        <v>191411</v>
+      </c>
+      <c r="G39" s="44">
+        <v>344916</v>
+      </c>
+      <c r="H39" s="40">
+        <v>2190</v>
+      </c>
+      <c r="I39" s="41">
+        <v>342727</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
-      <c r="B40" s="35">
-        <v>-119801</v>
+      <c r="B40" s="40">
+        <v>-87471</v>
       </c>
-      <c r="C40" s="36">
-        <v>-120619</v>
+      <c r="C40" s="41">
+        <v>-86422</v>
       </c>
-      <c r="D40" s="37">
-        <v>170423</v>
+      <c r="D40" s="42">
+        <v>190427</v>
       </c>
-      <c r="E40" s="38">
-        <v>2848</v>
+      <c r="E40" s="40">
+        <v>716</v>
       </c>
-      <c r="F40" s="39">
-        <v>167575</v>
+      <c r="F40" s="43">
+        <v>189711</v>
       </c>
-      <c r="G40" s="40">
-        <v>290224</v>
+      <c r="G40" s="44">
+        <v>277898</v>
       </c>
-      <c r="H40" s="38">
-        <v>2030</v>
+      <c r="H40" s="40">
+        <v>1765</v>
       </c>
-      <c r="I40" s="36">
-        <v>288194</v>
+      <c r="I40" s="41">
+        <v>276133</v>
       </c>
     </row>
     <row r="41" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
-      <c r="B41" s="35">
-        <v>-151950</v>
+      <c r="B41" s="40">
+        <v>-94536</v>
       </c>
-      <c r="C41" s="36">
-        <v>-151316</v>
+      <c r="C41" s="41">
+        <v>-93299</v>
       </c>
-      <c r="D41" s="37">
-        <v>192967</v>
+      <c r="D41" s="42">
+        <v>183767</v>
       </c>
-      <c r="E41" s="38">
-        <v>1556</v>
+      <c r="E41" s="40">
+        <v>663</v>
       </c>
-      <c r="F41" s="39">
-        <v>191411</v>
+      <c r="F41" s="43">
+        <v>183104</v>
       </c>
-      <c r="G41" s="40">
-        <v>344916</v>
+      <c r="G41" s="44">
+        <v>278303</v>
       </c>
-      <c r="H41" s="38">
-        <v>2190</v>
+      <c r="H41" s="40">
+        <v>1900</v>
       </c>
-      <c r="I41" s="36">
-        <v>342727</v>
+      <c r="I41" s="41">
+        <v>276403</v>
       </c>
     </row>
     <row r="42" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
-      <c r="B42" s="35">
-        <v>-87471</v>
+      <c r="B42" s="40">
+        <v>-86823</v>
       </c>
-      <c r="C42" s="36">
-        <v>-86422</v>
+      <c r="C42" s="41">
+        <v>-85391</v>
       </c>
-      <c r="D42" s="37">
-        <v>190427</v>
+      <c r="D42" s="42">
+        <v>180853</v>
       </c>
-      <c r="E42" s="38">
-        <v>716</v>
+      <c r="E42" s="40">
+        <v>726</v>
       </c>
-      <c r="F42" s="39">
-        <v>189711</v>
+      <c r="F42" s="43">
+        <v>180127</v>
       </c>
-      <c r="G42" s="40">
-        <v>277898</v>
+      <c r="G42" s="44">
+        <v>267675</v>
       </c>
-      <c r="H42" s="38">
-        <v>1765</v>
+      <c r="H42" s="40">
+        <v>2158</v>
       </c>
-      <c r="I42" s="36">
-        <v>276133</v>
+      <c r="I42" s="41">
+        <v>265518</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
-      <c r="B43" s="35">
-        <v>-94536</v>
+      <c r="B43" s="40">
+        <v>-117268</v>
       </c>
-      <c r="C43" s="36">
-        <v>-93299</v>
+      <c r="C43" s="41">
+        <v>-115980</v>
       </c>
-      <c r="D43" s="37">
-        <v>183767</v>
+      <c r="D43" s="42">
+        <v>177226</v>
       </c>
-      <c r="E43" s="38">
-        <v>663</v>
+      <c r="E43" s="40">
+        <v>991</v>
       </c>
-      <c r="F43" s="39">
-        <v>183104</v>
+      <c r="F43" s="43">
+        <v>176235</v>
       </c>
-      <c r="G43" s="40">
-        <v>278303</v>
+      <c r="G43" s="44">
+        <v>294494</v>
       </c>
-      <c r="H43" s="38">
-        <v>1900</v>
+      <c r="H43" s="40">
+        <v>2279</v>
       </c>
-      <c r="I43" s="36">
-        <v>276403</v>
+      <c r="I43" s="41">
+        <v>292215</v>
       </c>
     </row>
     <row r="44" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
-      <c r="B44" s="35">
-        <v>-86823</v>
+      <c r="B44" s="40">
+        <v>-84686</v>
       </c>
-      <c r="C44" s="36">
-        <v>-85391</v>
+      <c r="C44" s="41">
+        <v>-83296</v>
       </c>
-      <c r="D44" s="37">
-        <v>180853</v>
+      <c r="D44" s="42">
+        <v>180354</v>
       </c>
-      <c r="E44" s="38">
-        <v>726</v>
+      <c r="E44" s="40">
+        <v>802</v>
       </c>
-      <c r="F44" s="39">
-        <v>180127</v>
+      <c r="F44" s="43">
+        <v>179552</v>
       </c>
-      <c r="G44" s="40">
-        <v>267675</v>
+      <c r="G44" s="44">
+        <v>265041</v>
       </c>
-      <c r="H44" s="38">
-        <v>2158</v>
+      <c r="H44" s="40">
+        <v>2192</v>
       </c>
-      <c r="I44" s="36">
-        <v>265518</v>
+      <c r="I44" s="41">
+        <v>262849</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="34" t="s">
-        <v>19</v>
+    <row r="45" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="2" t="s">
+        <v>20</v>
       </c>
-      <c r="B45" s="35">
-        <v>-117268</v>
+      <c r="B45" s="40">
+        <v>-90743</v>
       </c>
-      <c r="C45" s="36">
-        <v>-115980</v>
+      <c r="C45" s="41">
+        <v>-89613</v>
       </c>
-      <c r="D45" s="37">
-        <v>177226</v>
+      <c r="D45" s="42">
+        <v>187595</v>
       </c>
-      <c r="E45" s="38">
-        <v>991</v>
+      <c r="E45" s="40">
+        <v>730</v>
       </c>
-      <c r="F45" s="39">
-        <v>176235</v>
+      <c r="F45" s="43">
+        <v>186865</v>
       </c>
-      <c r="G45" s="40">
-        <v>294494</v>
+      <c r="G45" s="44">
+        <v>278337</v>
       </c>
-      <c r="H45" s="38">
-        <v>2279</v>
+      <c r="H45" s="40">
+        <v>1860</v>
       </c>
-      <c r="I45" s="36">
-        <v>292215</v>
+      <c r="I45" s="41">
+        <v>276478</v>
       </c>
     </row>
     <row r="46" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
-      <c r="B46" s="35">
-        <v>-84686</v>
+      <c r="B46" s="40">
+        <v>-71954</v>
       </c>
-      <c r="C46" s="36">
-        <v>-83296</v>
+      <c r="C46" s="41">
+        <v>-71322</v>
       </c>
-      <c r="D46" s="37">
-        <v>180354</v>
+      <c r="D46" s="42">
+        <v>204314</v>
       </c>
-      <c r="E46" s="38">
-        <v>802</v>
+      <c r="E46" s="40">
+        <v>707</v>
       </c>
-      <c r="F46" s="39">
-        <v>179552</v>
+      <c r="F46" s="43">
+        <v>203607</v>
       </c>
-      <c r="G46" s="40">
-        <v>265041</v>
+      <c r="G46" s="44">
+        <v>276268</v>
       </c>
-      <c r="H46" s="38">
-        <v>2192</v>
+      <c r="H46" s="40">
+        <v>1339</v>
       </c>
-      <c r="I46" s="36">
-        <v>262849</v>
+      <c r="I46" s="41">
+        <v>274929</v>
       </c>
     </row>
     <row r="47" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
-      <c r="B47" s="35">
-        <v>-90743</v>
+      <c r="B47" s="40">
+        <v>-78474</v>
       </c>
-      <c r="C47" s="36">
-        <v>-89613</v>
+      <c r="C47" s="41">
+        <v>-77691</v>
       </c>
-      <c r="D47" s="37">
-        <v>187595</v>
+      <c r="D47" s="42">
+        <v>183853</v>
       </c>
-      <c r="E47" s="38">
-        <v>730</v>
+      <c r="E47" s="40">
+        <v>719</v>
       </c>
-      <c r="F47" s="39">
-        <v>186865</v>
+      <c r="F47" s="43">
+        <v>183135</v>
       </c>
-      <c r="G47" s="40">
-        <v>278337</v>
+      <c r="G47" s="44">
+        <v>262328</v>
       </c>
-      <c r="H47" s="38">
-        <v>1860</v>
+      <c r="H47" s="40">
+        <v>1502</v>
       </c>
-      <c r="I47" s="36">
-        <v>276478</v>
+      <c r="I47" s="41">
+        <v>260826</v>
       </c>
     </row>
     <row r="48" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="2" t="s">
+      <c r="A48" s="49" t="s">
+        <v>23</v>
+      </c>
+      <c r="B48" s="50">
+        <v>-103957</v>
+      </c>
+      <c r="C48" s="51">
+        <v>-103199</v>
+      </c>
+      <c r="D48" s="52">
+        <v>179815</v>
+      </c>
+      <c r="E48" s="50">
+        <v>779</v>
+      </c>
+      <c r="F48" s="53">
+        <v>179036</v>
+      </c>
+      <c r="G48" s="54">
+        <v>283772</v>
+      </c>
+      <c r="H48" s="50">
+        <v>1537</v>
+      </c>
+      <c r="I48" s="51">
+        <v>282235</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" ht="22.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A49" s="55" t="s">
         <v>27</v>
       </c>
-      <c r="B48" s="35">
-        <v>-71954</v>
-      </c>
-      <c r="C48" s="36">
-        <v>-71322</v>
-      </c>
-      <c r="D48" s="37">
-        <v>204314</v>
-      </c>
-      <c r="E48" s="38">
-        <v>707</v>
-      </c>
-      <c r="F48" s="39">
-        <v>203607</v>
-      </c>
-      <c r="G48" s="40">
-        <v>276268</v>
-      </c>
-      <c r="H48" s="38">
-        <v>1339</v>
-      </c>
-      <c r="I48" s="36">
-        <v>274929</v>
-      </c>
     </row>
-    <row r="49" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B49" s="35">
+    <row r="50" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B50" s="56">
         <v>-81207</v>
       </c>
-      <c r="C49" s="36">
+      <c r="C50" s="56">
         <v>-80425</v>
       </c>
-      <c r="D49" s="37">
+      <c r="D50" s="56">
         <v>182866</v>
       </c>
-      <c r="E49" s="38">
+      <c r="E50" s="56">
         <v>720</v>
       </c>
-      <c r="F49" s="39">
+      <c r="F50" s="56">
         <v>182146</v>
       </c>
-      <c r="G49" s="40">
+      <c r="G50" s="56">
         <v>264073</v>
       </c>
-      <c r="H49" s="38">
+      <c r="H50" s="56">
         <v>1502</v>
       </c>
-      <c r="I49" s="36">
+      <c r="I50" s="56">
         <v>262571</v>
       </c>
     </row>
-    <row r="50" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="41" t="s">
-        <v>24</v>
-      </c>
-      <c r="B50" s="42" t="s">
-        <v>28</v>
-      </c>
-      <c r="C50" s="43" t="s">
-        <v>28</v>
-      </c>
-      <c r="D50" s="44" t="s">
-        <v>28</v>
-      </c>
-      <c r="E50" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="F50" s="46" t="s">
-        <v>28</v>
-      </c>
-      <c r="G50" s="47" t="s">
-        <v>28</v>
-      </c>
-      <c r="H50" s="45" t="s">
-        <v>28</v>
-      </c>
-      <c r="I50" s="43" t="s">
+    <row r="51" spans="1:9" ht="25.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A51" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="51" spans="1:9" ht="22.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="53" t="s">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A52" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="52" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B52" s="54">
-        <v>-72043</v>
-      </c>
-      <c r="C52" s="54">
-        <v>-71407</v>
-      </c>
-      <c r="D52" s="54">
-        <v>203457</v>
-      </c>
-      <c r="E52" s="54">
-        <v>675</v>
-      </c>
-      <c r="F52" s="54">
-        <v>202783</v>
-      </c>
-      <c r="G52" s="54">
-        <v>275500</v>
-      </c>
-      <c r="H52" s="54">
-        <v>1310</v>
-      </c>
-      <c r="I52" s="54">
-        <v>274190</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" ht="22.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
+    <row r="53" spans="1:9" ht="22.25" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A5:A6"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
-  <pageSetup scale="58" firstPageNumber="14" orientation="portrait" useFirstPageNumber="1" r:id="rId1"/>
+  <pageSetup scale="57" firstPageNumber="14" orientation="portrait" useFirstPageNumber="1" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;C- &amp;P -</oddHeader>
   </headerFooter>

</xml_diff>